<commit_message>
Ajout moteur de scoring, endpoints API (questionnaire/reponses/resultats), génération rapport PDF enrichi
</commit_message>
<xml_diff>
--- a/backend/referentiel/data/referentiel_29_questions.xlsx
+++ b/backend/referentiel/data/referentiel_29_questions.xlsx
@@ -620,16 +620,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -665,6 +666,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>recommandation</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>ordre</t>
         </is>
       </c>
@@ -698,7 +704,12 @@
           <t>Art. 4</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Établir une politique de sécurité conforme à l'ISO 27001 (A.5.1.1)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -727,7 +738,12 @@
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Désigner un RSSI et définir ses responsabilités (ISO 27001 A.5.1.2)</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
         <v>2</v>
       </c>
     </row>
@@ -756,7 +772,12 @@
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Réaliser une analyse des risques selon ISO 27005 et NIST ID.RA-3</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -785,7 +806,12 @@
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Mettre en place un plan de sensibilisation annuel (NIST PR.AT-1)</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -818,7 +844,12 @@
           <t>Art. 24</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Formaliser une procédure de révocation des accès (NIST PR.AC-4)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -851,7 +882,12 @@
           <t>Art. 23</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Définir et appliquer une classification des données (ISO 27001 A.8.2.1)</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -884,7 +920,12 @@
           <t>Art. 36</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Inclure des clauses de sécurité dans les contrats (Loi 09-08 Art. 36)</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -913,7 +954,12 @@
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Implémenter un contrôle d'accès basé sur les rôles (RBAC)</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -946,7 +992,12 @@
           <t>Art. 23</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Appliquer une politique de mots de passe forte (complexité, rotation, MFA)</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
         <v>2</v>
       </c>
     </row>
@@ -979,7 +1030,12 @@
           <t>Art. 10</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Mettre en place un système de journalisation centralisé (SIEM)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1008,7 +1064,12 @@
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="n">
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Séparer les comptes administrateur et utilisateur (least privilege)</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1037,7 +1098,12 @@
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="n">
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Créer et maintenir un inventaire des comptes et droits</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1066,7 +1132,12 @@
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="n">
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Mettre en place une procédure stricte pour les comptes privilégiés</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1095,7 +1166,12 @@
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="n">
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Imposer l'authentification multifacteur pour tous les accès distants</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1124,7 +1200,12 @@
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="n">
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Sécuriser l'accès aux serveurs (badge, vidéo, HVAC)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1153,7 +1234,12 @@
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="n">
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Mettre en place des mesures de protection environnementale (détection incendie, onduleur/UPS, sauvegarde externalisée) — ISO 27001 A.11.1.4, NIST PR.PT-2</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1182,7 +1268,12 @@
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="n">
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Standardiser les systèmes et appliquer les patches (NIST PR.IP-1)</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1211,7 +1302,12 @@
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="n">
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Mettre en place pare-feu, VPN et segmentation réseau</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1244,7 +1340,12 @@
           <t>Art. 36</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Inclure des clauses de sécurité dans les contrats (Loi 09-08 Art. 36)</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1273,7 +1374,12 @@
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="n">
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Mettre en place un processus de gestion des vulnérabilités (NIST ID.RA-1)</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1306,7 +1412,12 @@
           <t>Art. 23</t>
         </is>
       </c>
-      <c r="G22" s="2" t="n">
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Contrôler l'usage des supports amovibles (chiffrement, antivirus)</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
         <v>7</v>
       </c>
     </row>
@@ -1335,7 +1446,12 @@
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="n">
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Adopter une approche DevSecOps (ISO 27001 A.8.25)</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1368,7 +1484,12 @@
           <t>Art. 39</t>
         </is>
       </c>
-      <c r="G24" s="2" t="n">
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Définir une procédure de gestion des incidents (ISO 27001 A.16.1.1)</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1397,7 +1518,12 @@
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="n">
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Élaborer un PCA/PRA avec RTO et RPO définis</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1430,7 +1556,12 @@
           <t>Art. 23</t>
         </is>
       </c>
-      <c r="G26" s="2" t="n">
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Mettre en place une stratégie de sauvegarde 3-2-1</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1459,7 +1590,12 @@
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="n">
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Documenter l'infrastructure et les processus (ISO 27001 A.12.1.1)</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
         <v>4</v>
       </c>
     </row>
@@ -1492,7 +1628,12 @@
           <t>Art. 5-10</t>
         </is>
       </c>
-      <c r="G28" s="2" t="n">
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Se mettre en conformité avec la loi 09-08 (Loi 09-08 Art. 5-10)</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1525,7 +1666,12 @@
           <t>Art. 39-40</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n">
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Mettre en place une procédure de notification des violations (72h)</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1554,7 +1700,12 @@
           <t>Art. 12</t>
         </is>
       </c>
-      <c r="G30" s="2" t="n">
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Réaliser des évaluations d'impact pour les traitements sensibles (Loi 09-08 Art. 12)</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
         <v>7</v>
       </c>
     </row>

</xml_diff>